<commit_message>
Add Cohen's d columns to Tables 2 and 3.
</commit_message>
<xml_diff>
--- a/output/tables/Table2_Main_Effects.xlsx
+++ b/output/tables/Table2_Main_Effects.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="143" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="181" uniqueCount="148">
   <si>
     <t>Table 2. Main-effects model predicting support for SNAP soft-drink/candy restrictions (N = 8715)</t>
   </si>
@@ -27,6 +27,9 @@
     <t>p</t>
   </si>
   <si>
+    <t>Cohen's d</t>
+  </si>
+  <si>
     <t>Self-reported soda overconsumption</t>
   </si>
   <si>
@@ -36,6 +39,9 @@
     <t>0.12</t>
   </si>
   <si>
+    <t>-0.02</t>
+  </si>
+  <si>
     <t>Perceived health risk of soda</t>
   </si>
   <si>
@@ -45,18 +51,27 @@
     <t>&lt;0.001</t>
   </si>
   <si>
+    <t>0.15</t>
+  </si>
+  <si>
     <t>Embarrassment when paying with SNAP</t>
   </si>
   <si>
     <t>-0.05 (-0.07, -0.03)</t>
   </si>
   <si>
+    <t>-0.03</t>
+  </si>
+  <si>
     <t>Perceived stigma of SNAP policies</t>
   </si>
   <si>
     <t>-0.27 (-0.36, -0.17)</t>
   </si>
   <si>
+    <t>-0.18</t>
+  </si>
+  <si>
     <t>SNAP participation past 3 months (W2 Q4)</t>
   </si>
   <si>
@@ -72,6 +87,9 @@
     <t>-0.54 (-0.64, -0.43)</t>
   </si>
   <si>
+    <t>-0.37</t>
+  </si>
+  <si>
     <t>age_bucket</t>
   </si>
   <si>
@@ -96,6 +114,9 @@
     <t>0.58</t>
   </si>
   <si>
+    <t>-0.30</t>
+  </si>
+  <si>
     <t xml:space="preserve">   35-44</t>
   </si>
   <si>
@@ -105,6 +126,9 @@
     <t>0.62</t>
   </si>
   <si>
+    <t>-0.27</t>
+  </si>
+  <si>
     <t xml:space="preserve">   45-54</t>
   </si>
   <si>
@@ -114,6 +138,9 @@
     <t>0.65</t>
   </si>
   <si>
+    <t>-0.25</t>
+  </si>
+  <si>
     <t xml:space="preserve">   55-64</t>
   </si>
   <si>
@@ -123,6 +150,9 @@
     <t>0.69</t>
   </si>
   <si>
+    <t>-0.21</t>
+  </si>
+  <si>
     <t xml:space="preserve">   65+</t>
   </si>
   <si>
@@ -132,6 +162,9 @@
     <t>0.85</t>
   </si>
   <si>
+    <t>-0.10</t>
+  </si>
+  <si>
     <t>gender</t>
   </si>
   <si>
@@ -144,6 +177,9 @@
     <t>0.15 (0.09, 0.21)</t>
   </si>
   <si>
+    <t>0.10</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Other</t>
   </si>
   <si>
@@ -153,6 +189,9 @@
     <t>0.29</t>
   </si>
   <si>
+    <t>0.11</t>
+  </si>
+  <si>
     <t>ethnicity</t>
   </si>
   <si>
@@ -174,13 +213,16 @@
     <t>-0.47 (-0.54, -0.40)</t>
   </si>
   <si>
+    <t>-0.32</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Hispanic/Latino</t>
   </si>
   <si>
     <t>0.07 (-0.02, 0.17)</t>
   </si>
   <si>
-    <t>0.10</t>
+    <t>0.05</t>
   </si>
   <si>
     <t>-0.24 (-0.39, -0.09)</t>
@@ -189,6 +231,9 @@
     <t>0.003</t>
   </si>
   <si>
+    <t>-0.16</t>
+  </si>
+  <si>
     <t>education</t>
   </si>
   <si>
@@ -204,6 +249,9 @@
     <t>0.25</t>
   </si>
   <si>
+    <t>-0.07</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Trade/Technical Degree</t>
   </si>
   <si>
@@ -213,6 +261,9 @@
     <t>0.39</t>
   </si>
   <si>
+    <t>-0.06</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Some College or university</t>
   </si>
   <si>
@@ -222,6 +273,9 @@
     <t>0.18</t>
   </si>
   <si>
+    <t>-0.08</t>
+  </si>
+  <si>
     <t xml:space="preserve">   2 year College Degree</t>
   </si>
   <si>
@@ -231,6 +285,9 @@
     <t>0.50</t>
   </si>
   <si>
+    <t>-0.04</t>
+  </si>
+  <si>
     <t xml:space="preserve">   4 year College Degree</t>
   </si>
   <si>
@@ -258,6 +315,9 @@
     <t>0.09</t>
   </si>
   <si>
+    <t>-0.12</t>
+  </si>
+  <si>
     <t>income</t>
   </si>
   <si>
@@ -273,6 +333,9 @@
     <t>0.02</t>
   </si>
   <si>
+    <t>0.07</t>
+  </si>
+  <si>
     <t xml:space="preserve">   $40k-60k</t>
   </si>
   <si>
@@ -291,6 +354,9 @@
     <t>0.30 (0.19, 0.42)</t>
   </si>
   <si>
+    <t>0.21</t>
+  </si>
+  <si>
     <t xml:space="preserve">   $100k-125k</t>
   </si>
   <si>
@@ -303,6 +369,9 @@
     <t>0.35 (0.22, 0.48)</t>
   </si>
   <si>
+    <t>0.24</t>
+  </si>
+  <si>
     <t>user_census_region_name</t>
   </si>
   <si>
@@ -315,7 +384,7 @@
     <t>0.06 (-0.04, 0.17)</t>
   </si>
   <si>
-    <t>0.24</t>
+    <t>0.04</t>
   </si>
   <si>
     <t xml:space="preserve">   South</t>
@@ -327,6 +396,9 @@
     <t>0.70</t>
   </si>
   <si>
+    <t>0.01</t>
+  </si>
+  <si>
     <t xml:space="preserve">   West</t>
   </si>
   <si>
@@ -366,6 +438,9 @@
     <t>0.75</t>
   </si>
   <si>
+    <t>-0.01</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Previously implemented but vacated</t>
   </si>
   <si>
@@ -378,7 +453,10 @@
     <t>0.24 (0.14, 0.34)</t>
   </si>
   <si>
-    <t>Note. OLS regression of support (1 = Strongly oppose to 5 = Strongly support) on all predictors and covariates, without predictor×SNAP interactions. Standard errors clustered by state (51 clusters). R-squared = 0.191. Unweighted; complete-case analysis. Multicollinearity was assessed with variance inflation factors before fitting (see 2_Main_Analysis log): all four psychological predictors and SNAP participation had VIF &lt; 1.5; larger VIFs reflect multi-category covariate dummy sets (e.g., age).</t>
+    <t>0.16</t>
+  </si>
+  <si>
+    <t>Note. OLS regression of support (1 = Strongly oppose to 5 = Strongly support) on all predictors and covariates, without predictor×SNAP interactions. Standard errors clustered by state (51 clusters). R-squared = 0.191. Cohen's d = b / SD(support), the change in support in outcome SD units associated with a 1-unit increase in a continuous predictor or with membership in a listed category versus the reference. Unweighted; complete-case analysis. Multicollinearity was assessed with variance inflation factors before fitting (see 2_Main_Analysis log): all four psychological predictors and SNAP participation had VIF &lt; 1.5; larger VIFs reflect multi-category covariate dummy sets (e.g., age).</t>
   </si>
 </sst>
 </file>
@@ -422,7 +500,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,534 +518,648 @@
       <c r="C2" t="s">
         <v>3</v>
       </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
         <v>11</v>
       </c>
-      <c r="C5" t="s">
-        <v>9</v>
+      <c r="D5" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>29</v>
+      </c>
+      <c r="D12" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C13" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="D13" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>36</v>
+      </c>
+      <c r="D14" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>32</v>
+        <v>40</v>
+      </c>
+      <c r="D15" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>44</v>
+      </c>
+      <c r="D16" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B17" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>48</v>
+      </c>
+      <c r="D17" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="B19" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="C20" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="D20" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="C21" t="s">
-        <v>45</v>
+        <v>57</v>
+      </c>
+      <c r="D21" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="B23" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="B24" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="C24" t="s">
-        <v>50</v>
+        <v>63</v>
+      </c>
+      <c r="D24" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="B25" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="C25" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="D25" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="B26" t="s">
+        <v>68</v>
+      </c>
+      <c r="C26" t="s">
         <v>54</v>
       </c>
-      <c r="C26" t="s">
-        <v>55</v>
+      <c r="D26" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="B27" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="C27" t="s">
-        <v>57</v>
+        <v>71</v>
+      </c>
+      <c r="D27" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="B29" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="B30" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="C30" t="s">
-        <v>62</v>
+        <v>77</v>
+      </c>
+      <c r="D30" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="B31" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="C31" t="s">
-        <v>65</v>
+        <v>81</v>
+      </c>
+      <c r="D31" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="B32" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="C32" t="s">
-        <v>68</v>
+        <v>85</v>
+      </c>
+      <c r="D32" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="B33" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="C33" t="s">
-        <v>71</v>
+        <v>89</v>
+      </c>
+      <c r="D33" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="B34" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="C34" t="s">
-        <v>74</v>
+        <v>93</v>
+      </c>
+      <c r="D34" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="B35" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="C35" t="s">
-        <v>77</v>
+        <v>96</v>
+      </c>
+      <c r="D35" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="B36" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="C36" t="s">
-        <v>80</v>
+        <v>99</v>
+      </c>
+      <c r="D36" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="B38" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="B39" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="C39" t="s">
-        <v>85</v>
+        <v>105</v>
+      </c>
+      <c r="D39" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="B40" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="C40" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="D40" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>88</v>
+        <v>109</v>
       </c>
       <c r="B41" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="C41" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="D41" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="B42" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="C42" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="D42" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="B43" t="s">
+        <v>115</v>
+      </c>
+      <c r="C43" t="s">
+        <v>11</v>
+      </c>
+      <c r="D43" t="s">
         <v>93</v>
-      </c>
-      <c r="C43" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="B44" t="s">
-        <v>95</v>
+        <v>117</v>
       </c>
       <c r="C44" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="D44" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="B46" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="B47" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C47" t="s">
-        <v>100</v>
+        <v>118</v>
+      </c>
+      <c r="D47" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="B48" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="C48" t="s">
-        <v>103</v>
+        <v>126</v>
+      </c>
+      <c r="D48" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>104</v>
+        <v>128</v>
       </c>
       <c r="B49" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="C49" t="s">
-        <v>106</v>
+        <v>130</v>
+      </c>
+      <c r="D49" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>107</v>
+        <v>131</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>108</v>
+        <v>132</v>
       </c>
       <c r="B51" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>109</v>
+        <v>133</v>
       </c>
       <c r="B52" t="s">
-        <v>110</v>
+        <v>134</v>
       </c>
       <c r="C52" t="s">
-        <v>111</v>
+        <v>135</v>
+      </c>
+      <c r="D52" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>112</v>
+        <v>136</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="B54" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="B55" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="C55" t="s">
-        <v>116</v>
+        <v>140</v>
+      </c>
+      <c r="D55" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="B56" t="s">
-        <v>118</v>
+        <v>143</v>
       </c>
       <c r="C56" t="s">
-        <v>80</v>
+        <v>99</v>
+      </c>
+      <c r="D56" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>119</v>
+        <v>144</v>
       </c>
       <c r="B57" t="s">
-        <v>120</v>
+        <v>145</v>
       </c>
       <c r="C57" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="D57" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>121</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Put Cohen's d before p-value in Tables 2 and 3.
</commit_message>
<xml_diff>
--- a/output/tables/Table2_Main_Effects.xlsx
+++ b/output/tables/Table2_Main_Effects.xlsx
@@ -24,36 +24,36 @@
     <t>b (95% CI)</t>
   </si>
   <si>
+    <t>Cohen's d</t>
+  </si>
+  <si>
     <t>p</t>
   </si>
   <si>
-    <t>Cohen's d</t>
-  </si>
-  <si>
     <t>Self-reported soda overconsumption</t>
   </si>
   <si>
     <t>-0.02 (-0.05, 0.01)</t>
   </si>
   <si>
+    <t>-0.02</t>
+  </si>
+  <si>
     <t>0.12</t>
   </si>
   <si>
-    <t>-0.02</t>
-  </si>
-  <si>
     <t>Perceived health risk of soda</t>
   </si>
   <si>
     <t>0.22 (0.19, 0.25)</t>
   </si>
   <si>
+    <t>0.15</t>
+  </si>
+  <si>
     <t>&lt;0.001</t>
   </si>
   <si>
-    <t>0.15</t>
-  </si>
-  <si>
     <t>Embarrassment when paying with SNAP</t>
   </si>
   <si>
@@ -111,60 +111,60 @@
     <t>-0.44 (-1.99, 1.12)</t>
   </si>
   <si>
+    <t>-0.30</t>
+  </si>
+  <si>
     <t>0.58</t>
   </si>
   <si>
-    <t>-0.30</t>
-  </si>
-  <si>
     <t xml:space="preserve">   35-44</t>
   </si>
   <si>
     <t>-0.39 (-1.95, 1.17)</t>
   </si>
   <si>
+    <t>-0.27</t>
+  </si>
+  <si>
     <t>0.62</t>
   </si>
   <si>
-    <t>-0.27</t>
-  </si>
-  <si>
     <t xml:space="preserve">   45-54</t>
   </si>
   <si>
     <t>-0.36 (-1.93, 1.21)</t>
   </si>
   <si>
+    <t>-0.25</t>
+  </si>
+  <si>
     <t>0.65</t>
   </si>
   <si>
-    <t>-0.25</t>
-  </si>
-  <si>
     <t xml:space="preserve">   55-64</t>
   </si>
   <si>
     <t>-0.31 (-1.88, 1.25)</t>
   </si>
   <si>
+    <t>-0.21</t>
+  </si>
+  <si>
     <t>0.69</t>
   </si>
   <si>
-    <t>-0.21</t>
-  </si>
-  <si>
     <t xml:space="preserve">   65+</t>
   </si>
   <si>
     <t>-0.15 (-1.72, 1.42)</t>
   </si>
   <si>
+    <t>-0.10</t>
+  </si>
+  <si>
     <t>0.85</t>
   </si>
   <si>
-    <t>-0.10</t>
-  </si>
-  <si>
     <t>gender</t>
   </si>
   <si>
@@ -186,12 +186,12 @@
     <t>0.16 (-0.14, 0.47)</t>
   </si>
   <si>
+    <t>0.11</t>
+  </si>
+  <si>
     <t>0.29</t>
   </si>
   <si>
-    <t>0.11</t>
-  </si>
-  <si>
     <t>ethnicity</t>
   </si>
   <si>
@@ -228,12 +228,12 @@
     <t>-0.24 (-0.39, -0.09)</t>
   </si>
   <si>
+    <t>-0.16</t>
+  </si>
+  <si>
     <t>0.003</t>
   </si>
   <si>
-    <t>-0.16</t>
-  </si>
-  <si>
     <t>education</t>
   </si>
   <si>
@@ -246,48 +246,48 @@
     <t>-0.10 (-0.27, 0.07)</t>
   </si>
   <si>
+    <t>-0.07</t>
+  </si>
+  <si>
     <t>0.25</t>
   </si>
   <si>
-    <t>-0.07</t>
-  </si>
-  <si>
     <t xml:space="preserve">   Trade/Technical Degree</t>
   </si>
   <si>
     <t>-0.08 (-0.28, 0.11)</t>
   </si>
   <si>
+    <t>-0.06</t>
+  </si>
+  <si>
     <t>0.39</t>
   </si>
   <si>
-    <t>-0.06</t>
-  </si>
-  <si>
     <t xml:space="preserve">   Some College or university</t>
   </si>
   <si>
     <t>-0.12 (-0.29, 0.06)</t>
   </si>
   <si>
+    <t>-0.08</t>
+  </si>
+  <si>
     <t>0.18</t>
   </si>
   <si>
-    <t>-0.08</t>
-  </si>
-  <si>
     <t xml:space="preserve">   2 year College Degree</t>
   </si>
   <si>
     <t>-0.06 (-0.25, 0.12)</t>
   </si>
   <si>
+    <t>-0.04</t>
+  </si>
+  <si>
     <t>0.50</t>
   </si>
   <si>
-    <t>-0.04</t>
-  </si>
-  <si>
     <t xml:space="preserve">   4 year College Degree</t>
   </si>
   <si>
@@ -312,12 +312,12 @@
     <t>-0.17 (-0.38, 0.03)</t>
   </si>
   <si>
+    <t>-0.12</t>
+  </si>
+  <si>
     <t>0.09</t>
   </si>
   <si>
-    <t>-0.12</t>
-  </si>
-  <si>
     <t>income</t>
   </si>
   <si>
@@ -330,12 +330,12 @@
     <t>0.10 (0.02, 0.19)</t>
   </si>
   <si>
+    <t>0.07</t>
+  </si>
+  <si>
     <t>0.02</t>
   </si>
   <si>
-    <t>0.07</t>
-  </si>
-  <si>
     <t xml:space="preserve">   $40k-60k</t>
   </si>
   <si>
@@ -393,12 +393,12 @@
     <t>0.02 (-0.08, 0.11)</t>
   </si>
   <si>
+    <t>0.01</t>
+  </si>
+  <si>
     <t>0.70</t>
   </si>
   <si>
-    <t>0.01</t>
-  </si>
-  <si>
     <t xml:space="preserve">   West</t>
   </si>
   <si>
@@ -435,10 +435,10 @@
     <t>-0.02 (-0.15, 0.11)</t>
   </si>
   <si>
+    <t>-0.01</t>
+  </si>
+  <si>
     <t>0.75</t>
-  </si>
-  <si>
-    <t>-0.01</t>
   </si>
   <si>
     <t xml:space="preserve">   Previously implemented but vacated</t>
@@ -558,10 +558,10 @@
         <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -572,10 +572,10 @@
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -599,10 +599,10 @@
         <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -626,10 +626,10 @@
         <v>28</v>
       </c>
       <c r="C12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" t="s">
         <v>29</v>
-      </c>
-      <c r="D12" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="13">
@@ -723,10 +723,10 @@
         <v>53</v>
       </c>
       <c r="C20" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="D20" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21">
@@ -764,10 +764,10 @@
         <v>62</v>
       </c>
       <c r="C24" t="s">
+        <v>54</v>
+      </c>
+      <c r="D24" t="s">
         <v>63</v>
-      </c>
-      <c r="D24" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="25">
@@ -778,10 +778,10 @@
         <v>65</v>
       </c>
       <c r="C25" t="s">
-        <v>11</v>
+        <v>66</v>
       </c>
       <c r="D25" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
     </row>
     <row r="26">
@@ -792,10 +792,10 @@
         <v>68</v>
       </c>
       <c r="C26" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" t="s">
         <v>54</v>
-      </c>
-      <c r="D26" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="27">
@@ -889,10 +889,10 @@
         <v>92</v>
       </c>
       <c r="C34" t="s">
+        <v>85</v>
+      </c>
+      <c r="D34" t="s">
         <v>93</v>
-      </c>
-      <c r="D34" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="35">
@@ -903,10 +903,10 @@
         <v>95</v>
       </c>
       <c r="C35" t="s">
+        <v>15</v>
+      </c>
+      <c r="D35" t="s">
         <v>96</v>
-      </c>
-      <c r="D35" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="36">
@@ -958,10 +958,10 @@
         <v>108</v>
       </c>
       <c r="C40" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D40" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41">
@@ -972,10 +972,10 @@
         <v>110</v>
       </c>
       <c r="C41" t="s">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="D41" t="s">
-        <v>93</v>
+        <v>12</v>
       </c>
     </row>
     <row r="42">
@@ -986,10 +986,10 @@
         <v>112</v>
       </c>
       <c r="C42" t="s">
-        <v>11</v>
+        <v>113</v>
       </c>
       <c r="D42" t="s">
-        <v>113</v>
+        <v>12</v>
       </c>
     </row>
     <row r="43">
@@ -1000,10 +1000,10 @@
         <v>115</v>
       </c>
       <c r="C43" t="s">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="D43" t="s">
-        <v>93</v>
+        <v>12</v>
       </c>
     </row>
     <row r="44">
@@ -1014,10 +1014,10 @@
         <v>117</v>
       </c>
       <c r="C44" t="s">
-        <v>11</v>
+        <v>118</v>
       </c>
       <c r="D44" t="s">
-        <v>118</v>
+        <v>12</v>
       </c>
     </row>
     <row r="45">
@@ -1041,10 +1041,10 @@
         <v>122</v>
       </c>
       <c r="C47" t="s">
+        <v>123</v>
+      </c>
+      <c r="D47" t="s">
         <v>118</v>
-      </c>
-      <c r="D47" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="48">
@@ -1069,10 +1069,10 @@
         <v>129</v>
       </c>
       <c r="C49" t="s">
+        <v>15</v>
+      </c>
+      <c r="D49" t="s">
         <v>130</v>
-      </c>
-      <c r="D49" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="50">
@@ -1096,10 +1096,10 @@
         <v>134</v>
       </c>
       <c r="C52" t="s">
+        <v>7</v>
+      </c>
+      <c r="D52" t="s">
         <v>135</v>
-      </c>
-      <c r="D52" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="53">
@@ -1137,10 +1137,10 @@
         <v>143</v>
       </c>
       <c r="C56" t="s">
-        <v>99</v>
+        <v>57</v>
       </c>
       <c r="D56" t="s">
-        <v>58</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57">
@@ -1151,10 +1151,10 @@
         <v>145</v>
       </c>
       <c r="C57" t="s">
-        <v>11</v>
+        <v>146</v>
       </c>
       <c r="D57" t="s">
-        <v>146</v>
+        <v>12</v>
       </c>
     </row>
     <row r="59">

</xml_diff>